<commit_message>
Finished archiving unused / old files and folders. Documentation is in "archiving information" folder. Rendered index.
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -374,30 +374,90 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>C:/AVIHAY/git/DCC-v3/notebooks/archive/preprocessing/charite/charite_loading_and_preprocessing.qmd</t>
+          <t>C:/AVIHAY/git/DCC-v3/scripts/archive/extract_ids_from_datastet_AC.R</t>
         </is>
       </c>
       <c r="B2">
-        <v>55</v>
+        <v>1</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>load(here("data", "raw", "charite", "master_od_screening_manual_check_2020_2023_v2.rda"))</t>
+          <t>load(here("data", "raw", "datastet", "archive", "all_results_unique.RData")) # load datastet output as an input to this code</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>C:/AVIHAY/git/DCC-v3/scripts/datasets_metadata_creation.R</t>
+          <t>C:/AVIHAY/git/DCC-v3/scripts/archive/get_files_and_their_mentions.R</t>
         </is>
       </c>
       <c r="B3">
-        <v>159</v>
+        <v>21</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>load(here("data", "raw", "charite", "master_od_screening_manual_check_2020_2023_v2.rda"))</t>
+          <t xml:space="preserve">  is_file_in_archive = str_detect(file_path, regex("archive", ignore_case = TRUE))</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>C:/AVIHAY/git/DCC-v3/scripts/archive/get_files_and_their_mentions.R</t>
+        </is>
+      </c>
+      <c r="B4">
+        <v>44</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        is_script_in_archive = str_detect(script_path, regex("archive", ignore_case = TRUE))</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>C:/AVIHAY/git/DCC-v3/scripts/archive/get_repo_folders_structure.R</t>
+        </is>
+      </c>
+      <c r="B5">
+        <v>8</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  "archive", ".Rproj.user", ".Rhistory", ".RData", ".Ruserdata",</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>C:/AVIHAY/git/DCC-v3/scripts/archive/sanity_check.R</t>
+        </is>
+      </c>
+      <c r="B6">
+        <v>19</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>g_teams &lt;- read_excel(here("data", "verification", "datastet_and_added_summarised", "archive", "dois_ids_grouped.xlsx"))</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>C:/AVIHAY/git/DCC-v3/scripts/archive/sanity_check.R</t>
+        </is>
+      </c>
+      <c r="B7">
+        <v>20</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>d_teams &lt;- read_excel(here("data", "verification", "datastet_and_added_summarised", "archive", "charite_dois_ids_distinct.xlsx"))</t>
         </is>
       </c>
     </row>

</xml_diff>